<commit_message>
Add DAL 2026Q1 results.
</commit_message>
<xml_diff>
--- a/airline_financial_data.xlsx
+++ b/airline_financial_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0f26b992e1a44723/Documents/School/UNCC/Personal Projects/US Airlines Financials Project/airline_financials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="459" documentId="8_{5FE741C9-A2F0-4D0A-8E2F-B83D587BBB42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E3FC9C9-A1B5-4890-BE0E-70BB459607B8}"/>
+  <xr:revisionPtr revIDLastSave="478" documentId="8_{5FE741C9-A2F0-4D0A-8E2F-B83D587BBB42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A09035F-7AF9-4242-89E7-4B1E2BD2855F}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{5CC2E0DD-0C2A-471D-BE08-E27D8B31800B}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="20">
   <si>
     <t>Year</t>
   </si>
@@ -956,7 +956,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95BF35CD-6CF2-4D2E-9294-3A1A732D8FBE}">
-  <dimension ref="A1:K201"/>
+  <dimension ref="A1:K205"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.5703125" bestFit="1" customWidth="1"/>
@@ -7555,6 +7555,71 @@
       </c>
       <c r="K201">
         <v>55000000</v>
+      </c>
+    </row>
+    <row r="202" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A202">
+        <v>2026</v>
+      </c>
+      <c r="B202">
+        <v>1</v>
+      </c>
+      <c r="C202" t="s">
+        <v>6</v>
+      </c>
+      <c r="D202">
+        <v>15854000000</v>
+      </c>
+      <c r="E202">
+        <v>12302000000</v>
+      </c>
+      <c r="F202">
+        <v>15353000000</v>
+      </c>
+      <c r="G202">
+        <v>-289000000</v>
+      </c>
+      <c r="H202">
+        <v>56470000000</v>
+      </c>
+      <c r="I202">
+        <v>69163000000</v>
+      </c>
+      <c r="K202">
+        <v>165000000</v>
+      </c>
+    </row>
+    <row r="203" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A203">
+        <v>2026</v>
+      </c>
+      <c r="B203">
+        <v>1</v>
+      </c>
+      <c r="C203" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="204" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A204">
+        <v>2026</v>
+      </c>
+      <c r="B204">
+        <v>1</v>
+      </c>
+      <c r="C204" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="205" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A205">
+        <v>2026</v>
+      </c>
+      <c r="B205">
+        <v>1</v>
+      </c>
+      <c r="C205" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adds 2026Q1 results and insights for all airlines. Adds long-term debt to quarterly results for the airlines that report it.
</commit_message>
<xml_diff>
--- a/airline_financial_data.xlsx
+++ b/airline_financial_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0f26b992e1a44723/Documents/School/UNCC/Personal Projects/US Airlines Financials Project/airline_financials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="478" documentId="8_{5FE741C9-A2F0-4D0A-8E2F-B83D587BBB42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A09035F-7AF9-4242-89E7-4B1E2BD2855F}"/>
+  <xr:revisionPtr revIDLastSave="614" documentId="8_{5FE741C9-A2F0-4D0A-8E2F-B83D587BBB42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF23B5FD-ADCB-4F8C-8465-89E03C8F0CCF}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{5CC2E0DD-0C2A-471D-BE08-E27D8B31800B}"/>
   </bookViews>
@@ -639,6 +639,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1035,6 +1039,9 @@
       <c r="I2">
         <v>65823000000</v>
       </c>
+      <c r="J2">
+        <v>21946000000</v>
+      </c>
       <c r="K2">
         <v>29000000</v>
       </c>
@@ -1131,6 +1138,9 @@
       <c r="I5">
         <v>72893000000</v>
       </c>
+      <c r="J5">
+        <v>21863000000</v>
+      </c>
       <c r="K5">
         <v>63000000</v>
       </c>
@@ -1163,6 +1173,9 @@
       <c r="I6">
         <v>68514000000</v>
       </c>
+      <c r="J6">
+        <v>8258000000</v>
+      </c>
       <c r="K6">
         <v>404000000</v>
       </c>
@@ -1227,6 +1240,9 @@
       <c r="I8">
         <v>75039000000</v>
       </c>
+      <c r="J8">
+        <v>22274000000</v>
+      </c>
       <c r="K8">
         <v>43000000</v>
       </c>
@@ -1259,6 +1275,9 @@
       <c r="I9">
         <v>72875000000</v>
       </c>
+      <c r="J9">
+        <v>7801000000</v>
+      </c>
       <c r="K9">
         <v>399000000</v>
       </c>
@@ -1323,6 +1342,9 @@
       <c r="I11">
         <v>68298000000</v>
       </c>
+      <c r="J11">
+        <v>20566000000</v>
+      </c>
       <c r="K11">
         <v>40000000</v>
       </c>
@@ -1355,6 +1377,9 @@
       <c r="I12">
         <v>62523000000</v>
       </c>
+      <c r="J12">
+        <v>7959000000</v>
+      </c>
       <c r="K12">
         <v>311000000</v>
       </c>
@@ -1387,6 +1412,9 @@
       <c r="I13">
         <v>68902000000</v>
       </c>
+      <c r="J13">
+        <v>12215000000</v>
+      </c>
       <c r="K13">
         <v>82000000</v>
       </c>
@@ -1524,6 +1552,9 @@
       <c r="I17">
         <v>66674000000</v>
       </c>
+      <c r="J17">
+        <v>20065000000</v>
+      </c>
       <c r="K17">
         <v>20000000</v>
       </c>
@@ -1556,6 +1587,9 @@
       <c r="I18">
         <v>62416000000</v>
       </c>
+      <c r="J18">
+        <v>7435000000</v>
+      </c>
       <c r="K18">
         <v>220000000</v>
       </c>
@@ -1620,6 +1654,9 @@
       <c r="I20">
         <v>72322000000</v>
       </c>
+      <c r="J20">
+        <v>21222000000</v>
+      </c>
       <c r="K20">
         <v>67000000</v>
       </c>
@@ -1652,6 +1689,9 @@
       <c r="I21">
         <v>71754000000</v>
       </c>
+      <c r="J21">
+        <v>7209000000</v>
+      </c>
       <c r="K21">
         <v>518000000</v>
       </c>
@@ -1716,6 +1756,9 @@
       <c r="I23">
         <v>75820000000</v>
       </c>
+      <c r="J23">
+        <v>21055000000</v>
+      </c>
       <c r="K23">
         <v>52000000</v>
       </c>
@@ -1748,6 +1791,9 @@
       <c r="I24">
         <v>75742000000</v>
       </c>
+      <c r="J24">
+        <v>7072000000</v>
+      </c>
       <c r="K24">
         <v>517000000</v>
       </c>
@@ -1812,6 +1858,9 @@
       <c r="I26">
         <v>70272000000</v>
       </c>
+      <c r="J26">
+        <v>20896000000</v>
+      </c>
       <c r="K26">
         <v>74000000</v>
       </c>
@@ -1844,6 +1893,9 @@
       <c r="I27">
         <v>65468000000</v>
       </c>
+      <c r="J27">
+        <v>8052000000</v>
+      </c>
       <c r="K27">
         <v>387000000</v>
       </c>
@@ -1876,6 +1928,9 @@
       <c r="I28">
         <v>71038000000</v>
       </c>
+      <c r="J28">
+        <v>13145000000</v>
+      </c>
       <c r="K28">
         <v>123000000</v>
       </c>
@@ -2013,6 +2068,9 @@
       <c r="I32">
         <v>62099000000</v>
       </c>
+      <c r="J32">
+        <v>21033000000</v>
+      </c>
       <c r="K32">
         <v>0</v>
       </c>
@@ -2045,6 +2103,9 @@
       <c r="I33">
         <v>58885000000</v>
       </c>
+      <c r="J33">
+        <v>11750000000</v>
+      </c>
       <c r="K33">
         <v>0</v>
       </c>
@@ -2109,6 +2170,9 @@
       <c r="I35">
         <v>17081000000</v>
       </c>
+      <c r="J35">
+        <v>28193000000</v>
+      </c>
       <c r="K35">
         <v>0</v>
       </c>
@@ -2141,6 +2205,9 @@
       <c r="I36">
         <v>10596000000</v>
       </c>
+      <c r="J36">
+        <v>18539000000</v>
+      </c>
       <c r="K36">
         <v>0</v>
       </c>
@@ -2205,6 +2272,9 @@
       <c r="I38">
         <v>30768000000</v>
       </c>
+      <c r="J38">
+        <v>29593000000</v>
+      </c>
       <c r="K38">
         <v>0</v>
       </c>
@@ -2237,6 +2307,9 @@
       <c r="I39">
         <v>28290000000</v>
       </c>
+      <c r="J39">
+        <v>28910000000</v>
+      </c>
       <c r="K39">
         <v>0</v>
       </c>
@@ -2301,6 +2374,9 @@
       <c r="I41">
         <v>33219000000</v>
       </c>
+      <c r="J41">
+        <v>29324000000</v>
+      </c>
       <c r="K41">
         <v>0</v>
       </c>
@@ -2333,6 +2409,9 @@
       <c r="I42">
         <v>36569000000</v>
       </c>
+      <c r="J42">
+        <v>26531000000</v>
+      </c>
       <c r="K42">
         <v>0</v>
       </c>
@@ -2365,6 +2444,9 @@
       <c r="I43">
         <v>30691000000</v>
       </c>
+      <c r="J43">
+        <v>24836000000</v>
+      </c>
       <c r="K43">
         <v>0</v>
       </c>
@@ -2502,6 +2584,9 @@
       <c r="I47">
         <v>37764000000</v>
       </c>
+      <c r="J47">
+        <v>36785000000</v>
+      </c>
       <c r="K47">
         <v>0</v>
       </c>
@@ -2534,6 +2619,9 @@
       <c r="I48">
         <v>40118000000</v>
       </c>
+      <c r="J48">
+        <v>24802000000</v>
+      </c>
       <c r="K48">
         <v>0</v>
       </c>
@@ -2598,6 +2686,9 @@
       <c r="I50">
         <v>54555000000</v>
       </c>
+      <c r="J50">
+        <v>36729000000</v>
+      </c>
       <c r="K50">
         <v>0</v>
       </c>
@@ -2630,6 +2721,9 @@
       <c r="I51">
         <v>48529000000</v>
       </c>
+      <c r="J51">
+        <v>25246000000</v>
+      </c>
       <c r="K51">
         <v>0</v>
       </c>
@@ -2694,6 +2788,9 @@
       <c r="I53">
         <v>61111000000</v>
       </c>
+      <c r="J53">
+        <v>35470000000</v>
+      </c>
       <c r="K53">
         <v>0</v>
       </c>
@@ -2726,6 +2823,9 @@
       <c r="I54">
         <v>54083000000</v>
       </c>
+      <c r="J54">
+        <v>24077000000</v>
+      </c>
       <c r="K54">
         <v>0</v>
       </c>
@@ -2790,6 +2890,9 @@
       <c r="I56">
         <v>61105000000</v>
       </c>
+      <c r="J56">
+        <v>35008000000</v>
+      </c>
       <c r="K56">
         <v>0</v>
       </c>
@@ -2822,6 +2925,9 @@
       <c r="I57">
         <v>51744000000</v>
       </c>
+      <c r="J57">
+        <v>23582000000</v>
+      </c>
       <c r="K57">
         <v>0</v>
       </c>
@@ -2854,6 +2960,9 @@
       <c r="I58">
         <v>54815000000</v>
       </c>
+      <c r="J58">
+        <v>30361000000</v>
+      </c>
       <c r="K58">
         <v>0</v>
       </c>
@@ -2991,6 +3100,9 @@
       <c r="I62">
         <v>59533000000</v>
       </c>
+      <c r="J62">
+        <v>34885000000</v>
+      </c>
       <c r="K62">
         <v>0</v>
       </c>
@@ -3023,6 +3135,9 @@
       <c r="I63">
         <v>51810000000</v>
       </c>
+      <c r="J63">
+        <v>22939000000</v>
+      </c>
       <c r="K63">
         <v>0</v>
       </c>
@@ -3087,6 +3202,9 @@
       <c r="I65">
         <v>66163000000</v>
       </c>
+      <c r="J65">
+        <v>34421000000</v>
+      </c>
       <c r="K65">
         <v>64000000</v>
       </c>
@@ -3119,6 +3237,9 @@
       <c r="I66">
         <v>58903000000</v>
       </c>
+      <c r="J66">
+        <v>21444000000</v>
+      </c>
       <c r="K66">
         <v>54000000</v>
       </c>
@@ -3183,6 +3304,9 @@
       <c r="I68">
         <v>68567000000</v>
       </c>
+      <c r="J68">
+        <v>33598000000</v>
+      </c>
       <c r="K68">
         <v>59000000</v>
       </c>
@@ -3215,6 +3339,9 @@
       <c r="I69">
         <v>63007000000</v>
       </c>
+      <c r="J69">
+        <v>19800000000</v>
+      </c>
       <c r="K69">
         <v>237000000</v>
       </c>
@@ -3279,6 +3406,9 @@
       <c r="I71">
         <v>65962000000</v>
       </c>
+      <c r="J71">
+        <v>31844000000</v>
+      </c>
       <c r="K71">
         <v>88000000</v>
       </c>
@@ -3311,6 +3441,9 @@
       <c r="I72">
         <v>59506000000</v>
       </c>
+      <c r="J72">
+        <v>19326000000</v>
+      </c>
       <c r="K72">
         <v>272000000</v>
       </c>
@@ -3343,6 +3476,9 @@
       <c r="I73">
         <v>64294000000</v>
       </c>
+      <c r="J73">
+        <v>28283000000</v>
+      </c>
       <c r="K73">
         <v>125000000</v>
       </c>
@@ -3480,6 +3616,9 @@
       <c r="I77">
         <v>65006000000</v>
       </c>
+      <c r="J77">
+        <v>31089000000</v>
+      </c>
       <c r="K77">
         <v>35000000</v>
       </c>
@@ -3512,6 +3651,9 @@
       <c r="I78">
         <v>61351000000</v>
       </c>
+      <c r="J78">
+        <v>18490000000</v>
+      </c>
       <c r="K78">
         <v>72000000</v>
       </c>
@@ -3576,6 +3718,9 @@
       <c r="I80">
         <v>69658000000</v>
       </c>
+      <c r="J80">
+        <v>30340000000</v>
+      </c>
       <c r="K80">
         <v>173000000</v>
       </c>
@@ -3608,6 +3753,9 @@
       <c r="I81">
         <v>68993000000</v>
       </c>
+      <c r="J81">
+        <v>16870000000</v>
+      </c>
       <c r="K81">
         <v>595000000</v>
       </c>
@@ -3672,6 +3820,9 @@
       <c r="I83">
         <v>73285000000</v>
       </c>
+      <c r="J83">
+        <v>29308000000</v>
+      </c>
       <c r="K83">
         <v>0</v>
       </c>
@@ -3704,6 +3855,9 @@
       <c r="I84">
         <v>73226000000</v>
       </c>
+      <c r="J84">
+        <v>16347000000</v>
+      </c>
       <c r="K84">
         <v>417000000</v>
       </c>
@@ -3768,6 +3922,9 @@
       <c r="I86">
         <v>69773000000</v>
       </c>
+      <c r="J86">
+        <v>28895000000</v>
+      </c>
       <c r="K86">
         <v>53000000</v>
       </c>
@@ -3800,6 +3957,9 @@
       <c r="I87">
         <v>68462000000</v>
       </c>
+      <c r="J87">
+        <v>15985000000</v>
+      </c>
       <c r="K87">
         <v>299000000</v>
       </c>
@@ -3832,6 +3992,9 @@
       <c r="I88">
         <v>73727000000</v>
       </c>
+      <c r="J88">
+        <v>25057000000</v>
+      </c>
       <c r="K88">
         <v>160000000</v>
       </c>
@@ -3969,6 +4132,9 @@
       <c r="I92">
         <v>70516000000</v>
       </c>
+      <c r="J92">
+        <v>27853000000</v>
+      </c>
       <c r="K92">
         <f>ROUND($K$179*((D92-F92)/($D$179-$F$179)),0)</f>
         <v>610559</v>
@@ -4002,6 +4168,9 @@
       <c r="I93">
         <v>65542000000</v>
       </c>
+      <c r="J93">
+        <v>15576000000</v>
+      </c>
       <c r="K93">
         <v>125000000</v>
       </c>
@@ -4066,6 +4235,9 @@
       <c r="I95">
         <v>75263000000</v>
       </c>
+      <c r="J95">
+        <v>27209000000</v>
+      </c>
       <c r="K95">
         <f>ROUND($K$179*((D95-F95)/($D$179-$F$179)),0)</f>
         <v>120716144</v>
@@ -4099,6 +4271,9 @@
       <c r="I96">
         <v>74656000000</v>
       </c>
+      <c r="J96">
+        <v>14084000000</v>
+      </c>
       <c r="K96">
         <v>519000000</v>
       </c>
@@ -4163,6 +4338,9 @@
       <c r="I98">
         <v>75665000000</v>
       </c>
+      <c r="J98">
+        <v>25848000000</v>
+      </c>
       <c r="K98">
         <f>ROUND($K$179*((D98-F98)/($D$179-$F$179)),0)</f>
         <v>7762816</v>
@@ -4196,6 +4374,9 @@
       <c r="I99">
         <v>76162000000</v>
       </c>
+      <c r="J99">
+        <v>13881000000</v>
+      </c>
       <c r="K99">
         <v>320000000</v>
       </c>
@@ -4366,7 +4547,7 @@
         <v>265657000000</v>
       </c>
       <c r="J104">
-        <v>16043000000</v>
+        <v>16196000000</v>
       </c>
       <c r="K104">
         <v>0</v>
@@ -5030,6 +5211,9 @@
       <c r="I123">
         <v>45219000000</v>
       </c>
+      <c r="J123">
+        <v>5075000000</v>
+      </c>
       <c r="K123">
         <v>18000000</v>
       </c>
@@ -5062,6 +5246,9 @@
       <c r="I124">
         <v>46250000000</v>
       </c>
+      <c r="J124">
+        <v>5065000000</v>
+      </c>
       <c r="K124">
         <v>31000000</v>
       </c>
@@ -5094,6 +5281,9 @@
       <c r="I125">
         <v>42248000000</v>
       </c>
+      <c r="J125">
+        <v>7974000000</v>
+      </c>
       <c r="K125">
         <v>0</v>
       </c>
@@ -5126,6 +5316,9 @@
       <c r="I126">
         <v>64341000000</v>
       </c>
+      <c r="J126">
+        <v>22829000000</v>
+      </c>
       <c r="K126">
         <v>31000000</v>
       </c>
@@ -5158,6 +5351,9 @@
       <c r="I127">
         <v>71743000000</v>
       </c>
+      <c r="J127">
+        <v>22525000000</v>
+      </c>
       <c r="K127">
         <v>94000000</v>
       </c>
@@ -5190,6 +5386,9 @@
       <c r="I128">
         <v>64582000000</v>
       </c>
+      <c r="J128">
+        <v>22217000000</v>
+      </c>
       <c r="K128">
         <v>70000000</v>
       </c>
@@ -5222,6 +5421,9 @@
       <c r="I129">
         <v>67355000000</v>
       </c>
+      <c r="J129">
+        <v>22511000000</v>
+      </c>
       <c r="K129">
         <v>47000000</v>
       </c>
@@ -5254,6 +5456,9 @@
       <c r="I130">
         <v>65064000000</v>
       </c>
+      <c r="J130">
+        <v>19134000000</v>
+      </c>
       <c r="K130">
         <v>73000000</v>
       </c>
@@ -5286,6 +5491,9 @@
       <c r="I131">
         <v>70751000000</v>
       </c>
+      <c r="J131">
+        <v>21131000000</v>
+      </c>
       <c r="K131">
         <v>98000000</v>
       </c>
@@ -5318,6 +5526,9 @@
       <c r="I132">
         <v>63751000000</v>
       </c>
+      <c r="J132">
+        <v>21545000000</v>
+      </c>
       <c r="K132">
         <v>86000000</v>
       </c>
@@ -5350,6 +5561,9 @@
       <c r="I133">
         <v>65683000000</v>
       </c>
+      <c r="J133">
+        <v>22489000000</v>
+      </c>
       <c r="K133">
         <v>57000000</v>
       </c>
@@ -5382,6 +5596,9 @@
       <c r="I134">
         <v>62791000000</v>
       </c>
+      <c r="J134">
+        <v>17638000000</v>
+      </c>
       <c r="K134">
         <v>0</v>
       </c>
@@ -5414,6 +5631,9 @@
       <c r="I135">
         <v>69401000000</v>
       </c>
+      <c r="J135">
+        <v>17152000000</v>
+      </c>
       <c r="K135">
         <v>0</v>
       </c>
@@ -5446,6 +5666,9 @@
       <c r="I136">
         <v>71092000000</v>
       </c>
+      <c r="J136">
+        <v>18849000000</v>
+      </c>
       <c r="K136">
         <v>0</v>
       </c>
@@ -5478,6 +5701,9 @@
       <c r="I137">
         <v>65453000000</v>
       </c>
+      <c r="J137">
+        <v>18330000000</v>
+      </c>
       <c r="K137">
         <v>0</v>
       </c>
@@ -5510,6 +5736,9 @@
       <c r="I138">
         <v>63392000000</v>
       </c>
+      <c r="J138">
+        <v>15244000000</v>
+      </c>
       <c r="K138">
         <v>0</v>
       </c>
@@ -5542,6 +5771,9 @@
       <c r="I139">
         <v>68090000000</v>
       </c>
+      <c r="J139">
+        <v>15205000000</v>
+      </c>
       <c r="K139">
         <v>0</v>
       </c>
@@ -5574,6 +5806,9 @@
       <c r="I140">
         <v>69120000000</v>
       </c>
+      <c r="J140">
+        <v>15651000000</v>
+      </c>
       <c r="K140">
         <v>0</v>
       </c>
@@ -5606,6 +5841,9 @@
       <c r="I141">
         <v>65053000000</v>
       </c>
+      <c r="J141">
+        <v>16196000000</v>
+      </c>
       <c r="K141">
         <v>0</v>
       </c>
@@ -5734,6 +5972,9 @@
       <c r="I145">
         <v>60060000000</v>
       </c>
+      <c r="J145">
+        <v>6295000000</v>
+      </c>
       <c r="K145">
         <v>262000000</v>
       </c>
@@ -5862,6 +6103,9 @@
       <c r="I149">
         <v>58715000000</v>
       </c>
+      <c r="J149">
+        <v>5999000000</v>
+      </c>
       <c r="K149">
         <v>193000000</v>
       </c>
@@ -5990,6 +6234,9 @@
       <c r="I153">
         <v>58199000000</v>
       </c>
+      <c r="J153">
+        <v>6531000000</v>
+      </c>
       <c r="K153">
         <v>380000000</v>
       </c>
@@ -6118,6 +6365,9 @@
       <c r="I157">
         <v>58029000000</v>
       </c>
+      <c r="J157">
+        <v>8188000000</v>
+      </c>
       <c r="K157">
         <v>262000000</v>
       </c>
@@ -6246,6 +6496,9 @@
       <c r="I161">
         <v>65028000000</v>
       </c>
+      <c r="J161">
+        <v>11703000000</v>
+      </c>
       <c r="K161">
         <v>73000000</v>
       </c>
@@ -6374,6 +6627,9 @@
       <c r="I165">
         <v>62518000000</v>
       </c>
+      <c r="J165">
+        <v>9918000000</v>
+      </c>
       <c r="K165">
         <v>145000000</v>
       </c>
@@ -6502,6 +6758,9 @@
       <c r="I169">
         <v>61304000000</v>
       </c>
+      <c r="J169">
+        <v>9673000000</v>
+      </c>
       <c r="K169">
         <v>146000000</v>
       </c>
@@ -6630,6 +6889,9 @@
       <c r="I173">
         <v>60213000000</v>
       </c>
+      <c r="J173">
+        <v>9953000000</v>
+      </c>
       <c r="K173">
         <v>54000000</v>
       </c>
@@ -6662,6 +6924,9 @@
       <c r="I174">
         <v>72035000000</v>
       </c>
+      <c r="J174">
+        <v>13546000000</v>
+      </c>
       <c r="K174">
         <v>425000000</v>
       </c>
@@ -6729,6 +6994,9 @@
       <c r="I176">
         <v>78298000000</v>
       </c>
+      <c r="J176">
+        <v>21680000000</v>
+      </c>
       <c r="K176">
         <v>294000000</v>
       </c>
@@ -6796,6 +7064,9 @@
       <c r="I178">
         <v>71503000000</v>
       </c>
+      <c r="J178">
+        <v>24617000000</v>
+      </c>
       <c r="K178">
         <f>ROUND($K$179*((D178-F178)/($D$179-$F$179)),0)</f>
         <v>98910482</v>
@@ -6864,6 +7135,9 @@
       <c r="I180">
         <v>43533000000</v>
       </c>
+      <c r="J180">
+        <v>5069000000</v>
+      </c>
       <c r="K180">
         <v>54000000</v>
       </c>
@@ -6931,6 +7205,9 @@
       <c r="I182">
         <v>68401000000</v>
       </c>
+      <c r="J182">
+        <v>12432000000</v>
+      </c>
       <c r="K182">
         <v>124000000</v>
       </c>
@@ -6995,6 +7272,9 @@
       <c r="I184">
         <v>69904000000</v>
       </c>
+      <c r="J184">
+        <v>24705000000</v>
+      </c>
       <c r="K184">
         <v>0</v>
       </c>
@@ -7027,6 +7307,9 @@
       <c r="I185">
         <v>41432000000</v>
       </c>
+      <c r="J185">
+        <v>4086000000</v>
+      </c>
       <c r="K185">
         <v>0</v>
       </c>
@@ -7059,6 +7342,9 @@
       <c r="I186">
         <v>77645000000</v>
       </c>
+      <c r="J186">
+        <v>12400000000</v>
+      </c>
       <c r="K186">
         <v>470000000</v>
       </c>
@@ -7123,6 +7409,9 @@
       <c r="I188">
         <v>77636000000</v>
       </c>
+      <c r="J188">
+        <v>24217000000</v>
+      </c>
       <c r="K188">
         <f>ROUND($K$201*(((D188-F188)/($D$201-$F$201))/(((D200-F200)/($D$201-$F$201))+((D188-F188)/($D$201-$F$201)))),0)</f>
         <v>39360025</v>
@@ -7156,6 +7445,9 @@
       <c r="I189">
         <v>46996000000</v>
       </c>
+      <c r="J189">
+        <v>4081000000</v>
+      </c>
       <c r="K189">
         <v>14000000</v>
       </c>
@@ -7188,6 +7480,9 @@
       <c r="I190">
         <v>79054000000</v>
       </c>
+      <c r="J190">
+        <v>12299000000</v>
+      </c>
       <c r="K190">
         <v>392000000</v>
       </c>
@@ -7252,6 +7547,9 @@
       <c r="I192">
         <v>77400000000</v>
       </c>
+      <c r="J192">
+        <v>24538000000</v>
+      </c>
       <c r="K192">
         <v>0</v>
       </c>
@@ -7284,6 +7582,9 @@
       <c r="I193">
         <v>45567000000</v>
       </c>
+      <c r="J193">
+        <v>4079000000</v>
+      </c>
       <c r="K193">
         <v>11000000</v>
       </c>
@@ -7316,6 +7617,9 @@
       <c r="I194">
         <v>72946000000</v>
       </c>
+      <c r="J194">
+        <v>11936000000</v>
+      </c>
       <c r="K194">
         <v>351000000</v>
       </c>
@@ -7383,6 +7687,9 @@
       <c r="I196">
         <v>83365000000</v>
       </c>
+      <c r="J196">
+        <v>17170000000</v>
+      </c>
       <c r="K196">
         <v>244000000</v>
       </c>
@@ -7450,6 +7757,9 @@
       <c r="I198">
         <v>46052000000</v>
       </c>
+      <c r="J198">
+        <v>4577000000</v>
+      </c>
       <c r="K198">
         <v>71000000</v>
       </c>
@@ -7517,6 +7827,9 @@
       <c r="I200">
         <v>74472000000</v>
       </c>
+      <c r="J200">
+        <v>24639000000</v>
+      </c>
       <c r="K200">
         <f>ROUND($K$201*(((D200-F200)/($D$201-$F$201))/(((D200-F200)/($D$201-$F$201))+((D188-F188)/($D$201-$F$201)))),0)</f>
         <v>15639975</v>
@@ -7585,6 +7898,9 @@
       <c r="I202">
         <v>69163000000</v>
       </c>
+      <c r="J202">
+        <v>10608000000</v>
+      </c>
       <c r="K202">
         <v>165000000</v>
       </c>
@@ -7599,6 +7915,27 @@
       <c r="C203" t="s">
         <v>7</v>
       </c>
+      <c r="D203">
+        <v>14608000000</v>
+      </c>
+      <c r="E203">
+        <v>13166000000</v>
+      </c>
+      <c r="F203">
+        <v>13611000000</v>
+      </c>
+      <c r="G203">
+        <v>699000000</v>
+      </c>
+      <c r="H203">
+        <v>63385000000</v>
+      </c>
+      <c r="I203">
+        <v>77698000000</v>
+      </c>
+      <c r="K203">
+        <v>59000000</v>
+      </c>
     </row>
     <row r="204" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A204">
@@ -7610,6 +7947,30 @@
       <c r="C204" t="s">
         <v>5</v>
       </c>
+      <c r="D204">
+        <v>13912000000</v>
+      </c>
+      <c r="E204">
+        <v>12495000000</v>
+      </c>
+      <c r="F204">
+        <v>13953000000</v>
+      </c>
+      <c r="G204">
+        <v>-382000000</v>
+      </c>
+      <c r="H204">
+        <v>58551000000</v>
+      </c>
+      <c r="I204">
+        <v>72009000000</v>
+      </c>
+      <c r="J204">
+        <v>22934000000</v>
+      </c>
+      <c r="K204">
+        <v>0</v>
+      </c>
     </row>
     <row r="205" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A205">
@@ -7620,6 +7981,30 @@
       </c>
       <c r="C205" t="s">
         <v>13</v>
+      </c>
+      <c r="D205">
+        <v>7249000000</v>
+      </c>
+      <c r="E205">
+        <v>6591000000</v>
+      </c>
+      <c r="F205">
+        <v>6919000000</v>
+      </c>
+      <c r="G205">
+        <v>330000000</v>
+      </c>
+      <c r="H205">
+        <v>31151000000</v>
+      </c>
+      <c r="I205">
+        <v>42049000000</v>
+      </c>
+      <c r="J205">
+        <v>4536000000</v>
+      </c>
+      <c r="K205">
+        <v>50000000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add DAL 2026Q2 results.
</commit_message>
<xml_diff>
--- a/airline_financial_data.xlsx
+++ b/airline_financial_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0f26b992e1a44723/Documents/School/UNCC/Personal Projects/US Airlines Financials Project/airline_financials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="614" documentId="8_{5FE741C9-A2F0-4D0A-8E2F-B83D587BBB42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF23B5FD-ADCB-4F8C-8465-89E03C8F0CCF}"/>
+  <xr:revisionPtr revIDLastSave="630" documentId="8_{5FE741C9-A2F0-4D0A-8E2F-B83D587BBB42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8275601D-DC47-427B-BA85-89E2A5276341}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{5CC2E0DD-0C2A-471D-BE08-E27D8B31800B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5CC2E0DD-0C2A-471D-BE08-E27D8B31800B}"/>
   </bookViews>
   <sheets>
     <sheet name="airline_financials" sheetId="2" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="20">
   <si>
     <t>Year</t>
   </si>
@@ -639,10 +639,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -960,23 +956,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95BF35CD-6CF2-4D2E-9294-3A1A732D8FBE}">
-  <dimension ref="A1:K205"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K209"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="17.140625" customWidth="1"/>
-    <col min="10" max="10" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="17.109375" customWidth="1"/>
+    <col min="10" max="10" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1011,7 +1007,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2018</v>
       </c>
@@ -1046,7 +1042,7 @@
         <v>29000000</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2018</v>
       </c>
@@ -1078,7 +1074,7 @@
         <v>188000000</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2018</v>
       </c>
@@ -1110,7 +1106,7 @@
         <v>17000000</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2018</v>
       </c>
@@ -1145,7 +1141,7 @@
         <v>63000000</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2018</v>
       </c>
@@ -1180,7 +1176,7 @@
         <v>404000000</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2018</v>
       </c>
@@ -1212,7 +1208,7 @@
         <v>108000000</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2018</v>
       </c>
@@ -1247,7 +1243,7 @@
         <v>43000000</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2018</v>
       </c>
@@ -1282,7 +1278,7 @@
         <v>399000000</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2018</v>
       </c>
@@ -1314,7 +1310,7 @@
         <v>127000000</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2018</v>
       </c>
@@ -1349,7 +1345,7 @@
         <v>40000000</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>2018</v>
       </c>
@@ -1384,7 +1380,7 @@
         <v>311000000</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>2018</v>
       </c>
@@ -1419,7 +1415,7 @@
         <v>82000000</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>2018</v>
       </c>
@@ -1454,7 +1450,7 @@
         <v>175000000</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>2018</v>
       </c>
@@ -1489,7 +1485,7 @@
         <v>1301000000</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>2018</v>
       </c>
@@ -1524,7 +1520,7 @@
         <v>334000000</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>2019</v>
       </c>
@@ -1559,7 +1555,7 @@
         <v>20000000</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>2019</v>
       </c>
@@ -1594,7 +1590,7 @@
         <v>220000000</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>2019</v>
       </c>
@@ -1626,7 +1622,7 @@
         <v>33000000</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>2019</v>
       </c>
@@ -1661,7 +1657,7 @@
         <v>67000000</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>2019</v>
       </c>
@@ -1696,7 +1692,7 @@
         <v>518000000</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>2019</v>
       </c>
@@ -1728,7 +1724,7 @@
         <v>161000000</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>2019</v>
       </c>
@@ -1763,7 +1759,7 @@
         <v>52000000</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>2019</v>
       </c>
@@ -1798,7 +1794,7 @@
         <v>517000000</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>2019</v>
       </c>
@@ -1830,7 +1826,7 @@
         <v>174000000</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>2019</v>
       </c>
@@ -1865,7 +1861,7 @@
         <v>74000000</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>2019</v>
       </c>
@@ -1900,7 +1896,7 @@
         <v>387000000</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>2019</v>
       </c>
@@ -1935,7 +1931,7 @@
         <v>123000000</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>2019</v>
       </c>
@@ -1970,7 +1966,7 @@
         <v>213000000</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>2019</v>
       </c>
@@ -2005,7 +2001,7 @@
         <v>1643000000</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>2019</v>
       </c>
@@ -2040,7 +2036,7 @@
         <v>491000000</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>2020</v>
       </c>
@@ -2075,7 +2071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>2020</v>
       </c>
@@ -2110,7 +2106,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>2020</v>
       </c>
@@ -2142,7 +2138,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>2020</v>
       </c>
@@ -2177,7 +2173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>2020</v>
       </c>
@@ -2212,7 +2208,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>2020</v>
       </c>
@@ -2244,7 +2240,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>2020</v>
       </c>
@@ -2279,7 +2275,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>2020</v>
       </c>
@@ -2314,7 +2310,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>2020</v>
       </c>
@@ -2346,7 +2342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>2020</v>
       </c>
@@ -2381,7 +2377,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>2020</v>
       </c>
@@ -2416,7 +2412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>2020</v>
       </c>
@@ -2451,7 +2447,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>2020</v>
       </c>
@@ -2486,7 +2482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>2020</v>
       </c>
@@ -2521,7 +2517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>2020</v>
       </c>
@@ -2556,7 +2552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>2021</v>
       </c>
@@ -2591,7 +2587,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>2021</v>
       </c>
@@ -2626,7 +2622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>2021</v>
       </c>
@@ -2658,7 +2654,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>2021</v>
       </c>
@@ -2693,7 +2689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>2021</v>
       </c>
@@ -2728,7 +2724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>2021</v>
       </c>
@@ -2760,7 +2756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>2021</v>
       </c>
@@ -2795,7 +2791,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>2021</v>
       </c>
@@ -2830,7 +2826,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>2021</v>
       </c>
@@ -2862,7 +2858,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>2021</v>
       </c>
@@ -2897,7 +2893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>2021</v>
       </c>
@@ -2932,7 +2928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>2021</v>
       </c>
@@ -2967,7 +2963,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>2021</v>
       </c>
@@ -3002,7 +2998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>2021</v>
       </c>
@@ -3037,7 +3033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>2021</v>
       </c>
@@ -3072,7 +3068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>2022</v>
       </c>
@@ -3107,7 +3103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>2022</v>
       </c>
@@ -3142,7 +3138,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>2022</v>
       </c>
@@ -3174,7 +3170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>2022</v>
       </c>
@@ -3209,7 +3205,7 @@
         <v>64000000</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>2022</v>
       </c>
@@ -3244,7 +3240,7 @@
         <v>54000000</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>2022</v>
       </c>
@@ -3276,7 +3272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>2022</v>
       </c>
@@ -3311,7 +3307,7 @@
         <v>59000000</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>2022</v>
       </c>
@@ -3346,7 +3342,7 @@
         <v>237000000</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>2022</v>
       </c>
@@ -3378,7 +3374,7 @@
         <v>8000000</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>2022</v>
       </c>
@@ -3413,7 +3409,7 @@
         <v>88000000</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>2022</v>
       </c>
@@ -3448,7 +3444,7 @@
         <v>272000000</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>2022</v>
       </c>
@@ -3483,7 +3479,7 @@
         <v>125000000</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>2022</v>
       </c>
@@ -3518,7 +3514,7 @@
         <v>211000000</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>2022</v>
       </c>
@@ -3553,7 +3549,7 @@
         <v>563000000</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>2022</v>
       </c>
@@ -3588,7 +3584,7 @@
         <v>133000000</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>2023</v>
       </c>
@@ -3623,7 +3619,7 @@
         <v>35000000</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>2023</v>
       </c>
@@ -3658,7 +3654,7 @@
         <v>72000000</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>2023</v>
       </c>
@@ -3690,7 +3686,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>2023</v>
       </c>
@@ -3725,7 +3721,7 @@
         <v>173000000</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>2023</v>
       </c>
@@ -3760,7 +3756,7 @@
         <v>595000000</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>2023</v>
       </c>
@@ -3792,7 +3788,7 @@
         <v>220000000</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>2023</v>
       </c>
@@ -3827,7 +3823,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>2023</v>
       </c>
@@ -3862,7 +3858,7 @@
         <v>417000000</v>
       </c>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>2023</v>
       </c>
@@ -3894,7 +3890,7 @@
         <v>301000000</v>
       </c>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>2023</v>
       </c>
@@ -3929,7 +3925,7 @@
         <v>53000000</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>2023</v>
       </c>
@@ -3964,7 +3960,7 @@
         <v>299000000</v>
       </c>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>2023</v>
       </c>
@@ -3999,7 +3995,7 @@
         <v>160000000</v>
       </c>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>2023</v>
       </c>
@@ -4034,7 +4030,7 @@
         <v>261000000</v>
       </c>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>2023</v>
       </c>
@@ -4069,7 +4065,7 @@
         <v>1383000000</v>
       </c>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>2023</v>
       </c>
@@ -4104,7 +4100,7 @@
         <v>681000000</v>
       </c>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>2024</v>
       </c>
@@ -4140,7 +4136,7 @@
         <v>610559</v>
       </c>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>2024</v>
       </c>
@@ -4175,7 +4171,7 @@
         <v>125000000</v>
       </c>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>2024</v>
       </c>
@@ -4207,7 +4203,7 @@
         <v>3000000</v>
       </c>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>2024</v>
       </c>
@@ -4243,7 +4239,7 @@
         <v>120716144</v>
       </c>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>2024</v>
       </c>
@@ -4278,7 +4274,7 @@
         <v>519000000</v>
       </c>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>2024</v>
       </c>
@@ -4310,7 +4306,7 @@
         <v>185000000</v>
       </c>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>2024</v>
       </c>
@@ -4346,7 +4342,7 @@
         <v>7762816</v>
       </c>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>2024</v>
       </c>
@@ -4381,7 +4377,7 @@
         <v>320000000</v>
       </c>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>2024</v>
       </c>
@@ -4413,7 +4409,7 @@
         <v>231000000</v>
       </c>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>2017</v>
       </c>
@@ -4448,7 +4444,7 @@
         <v>241000000</v>
       </c>
     </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>2016</v>
       </c>
@@ -4483,7 +4479,7 @@
         <v>314000000</v>
       </c>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>2015</v>
       </c>
@@ -4518,7 +4514,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>2014</v>
       </c>
@@ -4553,7 +4549,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>2017</v>
       </c>
@@ -4588,7 +4584,7 @@
         <v>1065000000</v>
       </c>
     </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>2016</v>
       </c>
@@ -4623,7 +4619,7 @@
         <v>1115000000</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>2015</v>
       </c>
@@ -4658,7 +4654,7 @@
         <v>1490000000</v>
       </c>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>2014</v>
       </c>
@@ -4693,7 +4689,7 @@
         <v>1085000000</v>
       </c>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>2017</v>
       </c>
@@ -4728,7 +4724,7 @@
         <v>349000000</v>
       </c>
     </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>2016</v>
       </c>
@@ -4763,7 +4759,7 @@
         <v>628000000</v>
       </c>
     </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>2015</v>
       </c>
@@ -4798,7 +4794,7 @@
         <v>698000000</v>
       </c>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>2014</v>
       </c>
@@ -4833,7 +4829,7 @@
         <v>235000000</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>2023</v>
       </c>
@@ -4868,7 +4864,7 @@
         <v>110000000</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>2022</v>
       </c>
@@ -4903,7 +4899,7 @@
         <v>127000000</v>
       </c>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>2021</v>
       </c>
@@ -4938,7 +4934,7 @@
         <v>230000000</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>2020</v>
       </c>
@@ -4973,7 +4969,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>2019</v>
       </c>
@@ -5008,7 +5004,7 @@
         <v>695000000</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>2018</v>
       </c>
@@ -5043,7 +5039,7 @@
         <v>580000000</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>2017</v>
       </c>
@@ -5078,7 +5074,7 @@
         <v>579000000</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>2016</v>
       </c>
@@ -5113,7 +5109,7 @@
         <v>645000000</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>2015</v>
       </c>
@@ -5148,7 +5144,7 @@
         <v>655000000</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>2014</v>
       </c>
@@ -5183,7 +5179,7 @@
         <v>374000000</v>
       </c>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>2024</v>
       </c>
@@ -5218,7 +5214,7 @@
         <v>18000000</v>
       </c>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A124">
         <v>2024</v>
       </c>
@@ -5253,7 +5249,7 @@
         <v>31000000</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>2024</v>
       </c>
@@ -5288,7 +5284,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>2017</v>
       </c>
@@ -5323,7 +5319,7 @@
         <v>31000000</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>2017</v>
       </c>
@@ -5358,7 +5354,7 @@
         <v>94000000</v>
       </c>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>2017</v>
       </c>
@@ -5393,7 +5389,7 @@
         <v>70000000</v>
       </c>
     </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>2017</v>
       </c>
@@ -5428,7 +5424,7 @@
         <v>47000000</v>
       </c>
     </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>2016</v>
       </c>
@@ -5463,7 +5459,7 @@
         <v>73000000</v>
       </c>
     </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>2016</v>
       </c>
@@ -5498,7 +5494,7 @@
         <v>98000000</v>
       </c>
     </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>2016</v>
       </c>
@@ -5533,7 +5529,7 @@
         <v>86000000</v>
       </c>
     </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>2016</v>
       </c>
@@ -5568,7 +5564,7 @@
         <v>57000000</v>
       </c>
     </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>2015</v>
       </c>
@@ -5603,7 +5599,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>2015</v>
       </c>
@@ -5638,7 +5634,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>2015</v>
       </c>
@@ -5673,7 +5669,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>2015</v>
       </c>
@@ -5708,7 +5704,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>2014</v>
       </c>
@@ -5743,7 +5739,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>2014</v>
       </c>
@@ -5778,7 +5774,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>2014</v>
       </c>
@@ -5813,7 +5809,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>2014</v>
       </c>
@@ -5848,7 +5844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>2017</v>
       </c>
@@ -5880,7 +5876,7 @@
         <v>151000000</v>
       </c>
     </row>
-    <row r="143" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>2017</v>
       </c>
@@ -5912,7 +5908,7 @@
         <v>338000000</v>
       </c>
     </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>2017</v>
       </c>
@@ -5944,7 +5940,7 @@
         <v>314000000</v>
       </c>
     </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A145">
         <v>2017</v>
       </c>
@@ -5979,7 +5975,7 @@
         <v>262000000</v>
       </c>
     </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A146">
         <v>2016</v>
       </c>
@@ -6011,7 +6007,7 @@
         <v>272000000</v>
       </c>
     </row>
-    <row r="147" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A147">
         <v>2016</v>
       </c>
@@ -6043,7 +6039,7 @@
         <v>324000000</v>
       </c>
     </row>
-    <row r="148" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>2016</v>
       </c>
@@ -6075,7 +6071,7 @@
         <v>326000000</v>
       </c>
     </row>
-    <row r="149" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A149">
         <v>2016</v>
       </c>
@@ -6110,7 +6106,7 @@
         <v>193000000</v>
       </c>
     </row>
-    <row r="150" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>2015</v>
       </c>
@@ -6142,7 +6138,7 @@
         <v>136000000</v>
       </c>
     </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>2015</v>
       </c>
@@ -6174,7 +6170,7 @@
         <v>411000000</v>
       </c>
     </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>2015</v>
       </c>
@@ -6206,7 +6202,7 @@
         <v>563000000</v>
       </c>
     </row>
-    <row r="153" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>2015</v>
       </c>
@@ -6241,7 +6237,7 @@
         <v>380000000</v>
       </c>
     </row>
-    <row r="154" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>2014</v>
       </c>
@@ -6273,7 +6269,7 @@
         <v>99000000</v>
       </c>
     </row>
-    <row r="155" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>2014</v>
       </c>
@@ -6305,7 +6301,7 @@
         <v>340000000</v>
       </c>
     </row>
-    <row r="156" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>2014</v>
       </c>
@@ -6337,7 +6333,7 @@
         <v>384000000</v>
       </c>
     </row>
-    <row r="157" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>2014</v>
       </c>
@@ -6372,7 +6368,7 @@
         <v>262000000</v>
       </c>
     </row>
-    <row r="158" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A158">
         <v>2017</v>
       </c>
@@ -6404,7 +6400,7 @@
         <v>28000000</v>
       </c>
     </row>
-    <row r="159" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A159">
         <v>2017</v>
       </c>
@@ -6436,7 +6432,7 @@
         <v>140000000</v>
       </c>
     </row>
-    <row r="160" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>2017</v>
       </c>
@@ -6468,7 +6464,7 @@
         <v>109000000</v>
       </c>
     </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A161">
         <v>2017</v>
       </c>
@@ -6503,7 +6499,7 @@
         <v>73000000</v>
       </c>
     </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>2016</v>
       </c>
@@ -6535,7 +6531,7 @@
         <v>94000000</v>
       </c>
     </row>
-    <row r="163" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A163">
         <v>2016</v>
       </c>
@@ -6567,7 +6563,7 @@
         <v>153000000</v>
       </c>
     </row>
-    <row r="164" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A164">
         <v>2016</v>
       </c>
@@ -6599,7 +6595,7 @@
         <v>235000000</v>
       </c>
     </row>
-    <row r="165" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A165">
         <v>2016</v>
       </c>
@@ -6634,7 +6630,7 @@
         <v>145000000</v>
       </c>
     </row>
-    <row r="166" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A166">
         <v>2015</v>
       </c>
@@ -6666,7 +6662,7 @@
         <v>100000000</v>
       </c>
     </row>
-    <row r="167" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A167">
         <v>2015</v>
       </c>
@@ -6698,7 +6694,7 @@
         <v>195000000</v>
       </c>
     </row>
-    <row r="168" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A168">
         <v>2015</v>
       </c>
@@ -6730,7 +6726,7 @@
         <v>257000000</v>
       </c>
     </row>
-    <row r="169" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A169">
         <v>2015</v>
       </c>
@@ -6765,7 +6761,7 @@
         <v>146000000</v>
       </c>
     </row>
-    <row r="170" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A170">
         <v>2014</v>
       </c>
@@ -6797,7 +6793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A171">
         <v>2014</v>
       </c>
@@ -6829,7 +6825,7 @@
         <v>78000000</v>
       </c>
     </row>
-    <row r="172" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A172">
         <v>2014</v>
       </c>
@@ -6861,7 +6857,7 @@
         <v>103000000</v>
       </c>
     </row>
-    <row r="173" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A173">
         <v>2014</v>
       </c>
@@ -6896,7 +6892,7 @@
         <v>54000000</v>
       </c>
     </row>
-    <row r="174" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A174">
         <v>2024</v>
       </c>
@@ -6931,7 +6927,7 @@
         <v>425000000</v>
       </c>
     </row>
-    <row r="175" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A175">
         <v>2024</v>
       </c>
@@ -6966,7 +6962,7 @@
         <v>1389000000</v>
       </c>
     </row>
-    <row r="176" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A176">
         <v>2024</v>
       </c>
@@ -7001,7 +6997,7 @@
         <v>294000000</v>
       </c>
     </row>
-    <row r="177" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A177">
         <v>2024</v>
       </c>
@@ -7036,7 +7032,7 @@
         <v>713000000</v>
       </c>
     </row>
-    <row r="178" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A178">
         <v>2024</v>
       </c>
@@ -7072,7 +7068,7 @@
         <v>98910482</v>
       </c>
     </row>
-    <row r="179" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A179">
         <v>2024</v>
       </c>
@@ -7107,7 +7103,7 @@
         <v>228000000</v>
       </c>
     </row>
-    <row r="180" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A180">
         <v>2024</v>
       </c>
@@ -7142,7 +7138,7 @@
         <v>54000000</v>
       </c>
     </row>
-    <row r="181" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A181">
         <v>2024</v>
       </c>
@@ -7177,7 +7173,7 @@
         <v>103000000</v>
       </c>
     </row>
-    <row r="182" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A182">
         <v>2025</v>
       </c>
@@ -7212,7 +7208,7 @@
         <v>124000000</v>
       </c>
     </row>
-    <row r="183" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A183">
         <v>2025</v>
       </c>
@@ -7244,7 +7240,7 @@
         <v>43000000</v>
       </c>
     </row>
-    <row r="184" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A184">
         <v>2025</v>
       </c>
@@ -7279,7 +7275,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A185">
         <v>2025</v>
       </c>
@@ -7314,7 +7310,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A186">
         <v>2025</v>
       </c>
@@ -7349,7 +7345,7 @@
         <v>470000000</v>
       </c>
     </row>
-    <row r="187" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A187">
         <v>2025</v>
       </c>
@@ -7381,7 +7377,7 @@
         <v>188000000</v>
       </c>
     </row>
-    <row r="188" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A188">
         <v>2025</v>
       </c>
@@ -7417,7 +7413,7 @@
         <v>39360025</v>
       </c>
     </row>
-    <row r="189" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A189">
         <v>2025</v>
       </c>
@@ -7452,7 +7448,7 @@
         <v>14000000</v>
       </c>
     </row>
-    <row r="190" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A190">
         <v>2025</v>
       </c>
@@ -7487,7 +7483,7 @@
         <v>392000000</v>
       </c>
     </row>
-    <row r="191" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A191">
         <v>2025</v>
       </c>
@@ -7519,7 +7515,7 @@
         <v>228000000</v>
       </c>
     </row>
-    <row r="192" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A192">
         <v>2025</v>
       </c>
@@ -7554,7 +7550,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A193">
         <v>2025</v>
       </c>
@@ -7589,7 +7585,7 @@
         <v>11000000</v>
       </c>
     </row>
-    <row r="194" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A194">
         <v>2025</v>
       </c>
@@ -7624,7 +7620,7 @@
         <v>351000000</v>
       </c>
     </row>
-    <row r="195" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A195">
         <v>2025</v>
       </c>
@@ -7659,7 +7655,7 @@
         <v>1337000000</v>
       </c>
     </row>
-    <row r="196" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A196">
         <v>2025</v>
       </c>
@@ -7694,7 +7690,7 @@
         <v>244000000</v>
       </c>
     </row>
-    <row r="197" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A197">
         <v>2025</v>
       </c>
@@ -7729,7 +7725,7 @@
         <v>704000000</v>
       </c>
     </row>
-    <row r="198" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A198">
         <v>2025</v>
       </c>
@@ -7764,7 +7760,7 @@
         <v>71000000</v>
       </c>
     </row>
-    <row r="199" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A199">
         <v>2025</v>
       </c>
@@ -7799,7 +7795,7 @@
         <v>97000000</v>
       </c>
     </row>
-    <row r="200" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A200">
         <v>2025</v>
       </c>
@@ -7835,7 +7831,7 @@
         <v>15639975</v>
       </c>
     </row>
-    <row r="201" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A201">
         <v>2025</v>
       </c>
@@ -7870,7 +7866,7 @@
         <v>55000000</v>
       </c>
     </row>
-    <row r="202" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A202">
         <v>2026</v>
       </c>
@@ -7905,7 +7901,7 @@
         <v>165000000</v>
       </c>
     </row>
-    <row r="203" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A203">
         <v>2026</v>
       </c>
@@ -7937,7 +7933,7 @@
         <v>59000000</v>
       </c>
     </row>
-    <row r="204" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A204">
         <v>2026</v>
       </c>
@@ -7972,7 +7968,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A205">
         <v>2026</v>
       </c>
@@ -8005,6 +8001,74 @@
       </c>
       <c r="K205">
         <v>50000000</v>
+      </c>
+    </row>
+    <row r="206" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A206">
+        <v>2026</v>
+      </c>
+      <c r="B206">
+        <v>2</v>
+      </c>
+      <c r="C206" t="s">
+        <v>6</v>
+      </c>
+      <c r="D206">
+        <v>19757000000</v>
+      </c>
+      <c r="E206">
+        <v>15607000000</v>
+      </c>
+      <c r="F206">
+        <v>17893000000</v>
+      </c>
+      <c r="G206">
+        <v>1604000000</v>
+      </c>
+      <c r="H206">
+        <v>66767000000</v>
+      </c>
+      <c r="I206">
+        <v>78694000000</v>
+      </c>
+      <c r="J206">
+        <v>10101000000</v>
+      </c>
+      <c r="K206">
+        <v>328000000</v>
+      </c>
+    </row>
+    <row r="207" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A207">
+        <v>2026</v>
+      </c>
+      <c r="B207">
+        <v>2</v>
+      </c>
+      <c r="C207" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="208" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A208">
+        <v>2026</v>
+      </c>
+      <c r="B208">
+        <v>2</v>
+      </c>
+      <c r="C208" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="209" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A209">
+        <v>2026</v>
+      </c>
+      <c r="B209">
+        <v>2</v>
+      </c>
+      <c r="C209" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -8015,13 +8079,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47E8CB36-28FD-4A01-8E6F-FAD97027E6F9}">
   <dimension ref="A1:E25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -8038,7 +8102,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2013</v>
       </c>
@@ -8055,7 +8119,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2014</v>
       </c>
@@ -8072,7 +8136,7 @@
         <v>1000000000</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2015</v>
       </c>
@@ -8089,7 +8153,7 @@
         <v>3600000000</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2016</v>
       </c>
@@ -8106,7 +8170,7 @@
         <v>4400000000</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2017</v>
       </c>
@@ -8123,7 +8187,7 @@
         <v>1600000000</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2018</v>
       </c>
@@ -8140,7 +8204,7 @@
         <v>800000000</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2019</v>
       </c>
@@ -8157,7 +8221,7 @@
         <v>1100000000</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2020</v>
       </c>
@@ -8174,7 +8238,7 @@
         <v>145000000</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2013</v>
       </c>
@@ -8191,7 +8255,7 @@
         <v>250000000</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2014</v>
       </c>
@@ -8208,7 +8272,7 @@
         <v>1100000000</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>2015</v>
       </c>
@@ -8225,7 +8289,7 @@
         <v>2200000000</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>2016</v>
       </c>
@@ -8242,7 +8306,7 @@
         <v>2600000000</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>2017</v>
       </c>
@@ -8259,7 +8323,7 @@
         <v>1700000000</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>2018</v>
       </c>
@@ -8276,7 +8340,7 @@
         <v>1600000000</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>2019</v>
       </c>
@@ -8293,7 +8357,7 @@
         <v>2000000000</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>2020</v>
       </c>
@@ -8310,7 +8374,7 @@
         <v>377620000</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>2013</v>
       </c>
@@ -8327,7 +8391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>2014</v>
       </c>
@@ -8344,7 +8408,7 @@
         <v>320000000</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>2015</v>
       </c>
@@ -8361,7 +8425,7 @@
         <v>1200000000</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>2016</v>
       </c>
@@ -8378,7 +8442,7 @@
         <v>2600000000</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>2017</v>
       </c>
@@ -8395,7 +8459,7 @@
         <v>1800000000</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>2018</v>
       </c>
@@ -8412,7 +8476,7 @@
         <v>1200000000</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>2019</v>
       </c>
@@ -8429,7 +8493,7 @@
         <v>1600000000</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>2020</v>
       </c>
@@ -8454,16 +8518,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{490D347E-B079-4188-B046-54C6AF8BB324}">
   <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.85546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="4.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.88671875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -8480,7 +8544,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2020</v>
       </c>
@@ -8497,7 +8561,7 @@
         <v>1901355562.5899999</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2021</v>
       </c>
@@ -8514,7 +8578,7 @@
         <v>1082205377.28</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2020</v>
       </c>
@@ -8531,7 +8595,7 @@
         <v>158535000</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2021</v>
       </c>
@@ -8548,7 +8612,7 @@
         <v>83433000</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2020</v>
       </c>
@@ -8565,7 +8629,7 @@
         <v>2293578491.5</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2021</v>
       </c>

</xml_diff>